<commit_message>
Add support for one-off schedule exceptions
- Introduced a new argument `--exceptions-filename` in the CLI for specifying a file containing one-off schedule events.
- Updated `CourseSiteConfig` to include `exceptions_filename` and initialized it to "exceptions.md".
- Implemented `parse_exception_events` function to read and process exceptions from the specified file.
- Modified `build_week_table` to include additional events from the exceptions in the weekly schedule.
- Updated calendar generation functions to incorporate exception events.
- Enhanced documentation in `calendar_schedule.md` and `weekly_schedule.md` to reflect the inclusion of exceptions.
- Created a new `exceptions.md` template for instructors to define one-off events.
</commit_message>
<xml_diff>
--- a/materials/generated_outputs/Weekly Schedules.xlsx
+++ b/materials/generated_outputs/Weekly Schedules.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -432,7 +432,8 @@
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,6 +464,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Additional Events</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Instructor Flags</t>
         </is>
       </c>
@@ -487,7 +493,8 @@
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Lab 1: Prerequisite may be same-day: M1.L01: Classify and Analyze Variables (first covered Lecture 2) | Lab 1: Prerequisite may be same-day: M1.L02: Evaluate Study Design and Its Implications (first covered Lecture 2) | Lab 1: Prerequisite may be same-day: M1.L03: Use R for Data Management and Exploration (first covered Lecture 2)</t>
         </is>
@@ -517,7 +524,8 @@
           <t>Lab 2: Lab1 in-lab activity submission | Tutorial 1 | Tutorial 2 (pre-lab for lab2)</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Lecture 3: Near Labor Day Holiday, Classes Suspended</t>
         </is>
@@ -548,6 +556,7 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -574,6 +583,7 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -600,6 +610,7 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -626,6 +637,7 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -651,7 +663,8 @@
           <t>Project1-2: Lab5 in-lab activity submission</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
         <is>
           <t>Lecture 16: Near Indigenous People's Day Holiday, Classes Suspended | Lecture 16: Substitute a Monday schedule of classes | Quiz 2: Near Indigenous People's Day Holiday, Classes Suspended | Quiz 2: Near Substitute a Monday schedule of classes</t>
         </is>
@@ -681,7 +694,8 @@
           <t>Project2-1: Project1 Video</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>Project2-1: Prerequisite not yet covered: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | Project2-1: Prerequisite not yet covered: M4.L01: Inference for a Difference in Proportions (first covered Lecture 21) | Project2-1: Prerequisite not yet covered: M4.L02: Conduct and Interpret Chi-Square Tests (first covered Lecture 22) | Project2-1: Prerequisite not yet covered: M4.L04: Conduct and Interpret t-Tests (first covered Lecture 24) | Project2-1: Prerequisite not yet covered: M4.L05: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
         </is>
@@ -711,7 +725,8 @@
           <t>Lab 6: Lab6 in-lab activity submission | Tutorial 6 (pre-lab for lab6) | Project2 Outline</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>Lab 6: Prerequisite not yet covered: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28)</t>
         </is>
@@ -741,7 +756,8 @@
           <t>Project2-2: Lab6 in-lab activity submission</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
         <is>
           <t>Quiz 3: Prerequisite not yet covered: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | Project2-2: Prerequisite not yet covered: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | Project2-2: Prerequisite not yet covered: M4.L05: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
         </is>
@@ -771,7 +787,8 @@
           <t>Project2-3: Project2 Progress Report</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>Project2-3: Prerequisite may be same-day: M3.L05: Distinguish Statistical vs. Practical Significance (first covered Lecture 28) | Project2-3: Prerequisite may be same-day: M4.L05: Explain Hypothesis Testing and Its Limitations (first covered Lecture 28)</t>
         </is>
@@ -801,7 +818,8 @@
           <t>Lab 7: Project2 writeup | Tutorial 7 (pre-lab for lab7)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
         <is>
           <t>Lab 7: Prerequisite may be same-day: M5.L03: Comparing Bayesian and Frequentist Approaches (first covered Lecture 31)</t>
         </is>
@@ -831,7 +849,8 @@
           <t>Lab 8: Project2 Resubmission</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>Lecture 32: Near Thanksgiving Recess | Lab 8: Near Thanksgiving Recess | Lab 8: Classes Resume | Lab 8: Missing prerequisite metadata: add learning-objective tags for Lab 8</t>
         </is>
@@ -853,7 +872,8 @@
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>Quiz 4: Near Thanksgiving Recess | Quiz 4: Classes Resume | Lecture 33: Near Classes Resume</t>
         </is>
@@ -875,7 +895,8 @@
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>Quiz 5: Near Last Day of Classes; Second Seven-Week Session Ends | Quiz 5: Near Study Period | Lecture 36: Last Day of Classes; Second Seven-Week Session Ends | Lecture 36: Near Study Period</t>
         </is>

</xml_diff>

<commit_message>
Add support for instructor-defined one-off events via exceptions.md.
- Add exceptions.md input table for custom calendar/schedule events
- Parse date-based exception rows into generated calendar and ICS outputs
- Add an Additional Events column to weekly schedule outputs
- Support custom exception input filename in the CLI
- Document exception event format and add an example row
- Add fallback calendar styling for custom event types
</commit_message>
<xml_diff>
--- a/materials/generated_outputs/Weekly Schedules.xlsx
+++ b/materials/generated_outputs/Weekly Schedules.xlsx
@@ -432,7 +432,7 @@
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -636,7 +636,11 @@
           <t>Lab 5: Lab4 in-lab activity submission | Tutorial 5 (pre-lab for lab5)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Midterm Review, 5:00PM-6:00PM</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
docs: modify learning objectives classification
- Clarify Core and Auxiliary objective counts
- Distinguish project assessment tags from objectives
- Document 22 Core and 11 Auxiliary objectives
</commit_message>
<xml_diff>
--- a/materials/generated_outputs/Weekly Schedules.xlsx
+++ b/materials/generated_outputs/Weekly Schedules.xlsx
@@ -430,7 +430,7 @@
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="37" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
@@ -489,7 +489,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Lab 1 (Lecture 1)</t>
+          <t>Lab 1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -516,7 +516,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Lab 2 (Lecture 3)</t>
+          <t>Lab 2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lab 3 (Lecture 6)</t>
+          <t>Lab 3</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Lab 4 (Lecture 11)</t>
+          <t>Lab 4</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lab 5 (Lecture 14)</t>
+          <t>Lab 5</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Lab 6 (Lecture 22)</t>
+          <t>Lab 6</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Lab 7 (Lecture 30)</t>
+          <t>Lab 7</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">

</xml_diff>

<commit_message>
docs(fall2026): sync syllabus, schedule, and Lecture 1
Update the syllabus inputs (staff office
hours, 18 core objectives, GenAI policy, homework and materials rules)
The document can be regenerated instead of maintained by hand.

Teach the generator the last things it couldn't reproduce: per-week
Weekly Plan overrides from the new syllabus_weekly_plan.md, the
reference table styling, and {{...}} raw-LaTeX passthrough.

Move Homework 1 to Tuesday and lab deliverables to Friday 9:00AM, and
bring Lecture 1 in line: handouts without solutions, named TFs and LAs,
lecture-time quizzes, and tutorials due before each lab.
</commit_message>
<xml_diff>
--- a/materials/generated_outputs/Weekly Schedules.xlsx
+++ b/materials/generated_outputs/Weekly Schedules.xlsx
@@ -492,7 +492,11 @@
           <t>Lab 1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Lab 1: Lab1 in-lab activity submission | Tutorial 1</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>

</xml_diff>